<commit_message>
docs: aplicar 22 correcciones de lectura crítica (vocabulario, coherencia interna, suavizado de menciones al profesor)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -720,6 +720,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="26">
       <c r="A4" s="23" t="inlineStr">
         <is>
@@ -768,6 +769,8 @@
       </c>
       <c r="H5" s="24" t="n"/>
     </row>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8" ht="15.75" customHeight="1" s="26">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -840,7 +843,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Cualquier rol</t>
+          <t>Cualquier usuario autenticado</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1200,7 +1203,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Cualquier autorizado</t>
+          <t>Residente, supervisión o contratista</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -1440,7 +1443,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Supervisión + Residencia</t>
+          <t>Supervisión y residencia</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -1640,7 +1643,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Contratista + Finanzas</t>
+          <t>Contratista y finanzas</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -1937,8 +1940,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2442,8 +2445,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2685,8 +2688,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3190,8 +3193,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3433,8 +3436,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3938,8 +3941,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4181,8 +4184,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4690,8 +4693,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4933,8 +4936,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5000,6 +5003,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="26">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -5015,7 +5019,7 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>contratista y Finanzas</t>
+          <t>contratista y finanzas</t>
         </is>
       </c>
       <c r="C6" s="32" t="n"/>
@@ -5049,6 +5053,7 @@
       <c r="C8" s="32" t="n"/>
       <c r="D8" s="24" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="26">
       <c r="A10" s="30" t="inlineStr">
         <is>
@@ -5128,6 +5133,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="26">
       <c r="A16" s="30" t="inlineStr">
         <is>
@@ -5438,8 +5444,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6336,8 +6342,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6579,8 +6585,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6822,8 +6828,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7065,8 +7071,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7308,8 +7314,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7551,8 +7557,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs(auditoria-legal): agregar reportes de verificacion y cobertura LOPSRM/RLOPSRM/LFD, matriz de permisos, PDFs de ley; citar art. 53 (residencia) y art. 118 RLOPSRM (CA-3 HU-12)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -720,7 +720,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="26">
       <c r="A4" s="23" t="inlineStr">
         <is>
@@ -769,8 +768,6 @@
       </c>
       <c r="H5" s="24" t="n"/>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8" ht="15.75" customHeight="1" s="26">
       <c r="A8" s="29" t="inlineStr">
         <is>
@@ -1940,8 +1937,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2445,8 +2442,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2688,8 +2685,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2873,7 +2870,7 @@
       </c>
       <c r="B14" s="34" t="inlineStr">
         <is>
-          <t>El sistema bloquea la integración cuando una cantidad por concepto excede la cantidad contratada en el catálogo.</t>
+          <t>El sistema bloquea la integración cuando una cantidad por concepto excede la cantidad contratada en el catálogo (art. 118 RLOPSRM: los trabajos por mayor valor sin orden escrita no son pagables).</t>
         </is>
       </c>
       <c r="C14" s="24" t="n"/>
@@ -3193,8 +3190,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3436,8 +3433,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3546,7 +3543,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>decidir sobre la estimación con evidencia completa y dentro de los plazos de los arts. 54 LOPSRM y 133 RLOPSRM</t>
+          <t>decidir sobre la estimación con evidencia completa, en ejercicio de la responsabilidad de la residencia sobre la revisión y aprobación (art. 53 LOPSRM), y dentro de los plazos de los arts. 54 LOPSRM y 133 RLOPSRM</t>
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
@@ -3941,8 +3938,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4184,8 +4181,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4693,8 +4690,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4936,8 +4933,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5003,7 +5000,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="26">
       <c r="A5" s="30" t="inlineStr">
         <is>
@@ -5053,7 +5049,6 @@
       <c r="C8" s="32" t="n"/>
       <c r="D8" s="24" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="26">
       <c r="A10" s="30" t="inlineStr">
         <is>
@@ -5133,7 +5128,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="26">
       <c r="A16" s="30" t="inlineStr">
         <is>
@@ -5444,8 +5438,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6342,8 +6336,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6585,8 +6579,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6828,8 +6822,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7071,8 +7065,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7314,8 +7308,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7557,8 +7551,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs(cobertura-legal): citar arts. 52 Bis (bitacora ley), 143 (amortizacion), 59 Bis (modif >50%), 55 (gastos financieros), 130 (tipos de estimacion) en HU y matriz de trazabilidad
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -1804,7 +1804,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>habilitar el registro formal de eventos del contrato conforme al art. 46 último párrafo LOPSRM y al art. 122 RLOPSRM</t>
+          <t>habilitar el registro formal de eventos del contrato conforme al art. 46 último párrafo y al art. 52 Bis LOPSRM (bitácora electrónica obligatoria), reglamentados por el art. 122 RLOPSRM</t>
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
@@ -1937,8 +1937,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2442,8 +2442,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2685,8 +2685,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>La carátula calcula automáticamente anticipo amortizado, retenciones legales (5 al millar) y deductivas por penalizaciones según el contrato.</t>
+          <t>La carátula calcula automáticamente el anticipo amortizado (proporcional, art. 143 RLOPSRM), las retenciones legales (5 al millar, art. 191 LFD) y las deductivas por penalizaciones según el contrato.</t>
         </is>
       </c>
       <c r="C13" s="24" t="n"/>
@@ -3190,8 +3190,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>ver la trazabilidad completa del ciclo de cobro del contrato, incluyendo versiones rechazadas</t>
+          <t>ver la trazabilidad completa del ciclo de cobro del contrato, incluyendo versiones rechazadas, conforme a los tipos de estimación reconocidos en el art. 130 RLOPSRM</t>
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
@@ -3433,8 +3433,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3938,8 +3938,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4181,8 +4181,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4690,8 +4690,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4933,8 +4933,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>no perder el plazo de pago y dejar evidencia de la suficiencia presupuestal verificada</t>
+          <t>no perder el plazo de pago y dejar evidencia de la suficiencia presupuestal verificada, considerando que el incumplimiento del plazo de pago genera gastos financieros a cargo de la dependencia (art. 55 LOPSRM)</t>
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
@@ -5438,8 +5438,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6336,8 +6336,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>documentar formalmente los cambios al contrato conforme al art. 59 LOPSRM y poder consultar qué cambió, cuándo y por qué</t>
+          <t>documentar formalmente los cambios al contrato conforme a los arts. 59 y 59 Bis LOPSRM (este último cuando la modificación supera el 50% del importe o del plazo) y poder consultar qué cambió, cuándo y por qué</t>
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
@@ -6579,8 +6579,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6822,8 +6822,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7065,8 +7065,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7308,8 +7308,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7551,8 +7551,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs(coherencia): alinear tipos de nota HU-09 al art. 125 RLOPSRM; reformular menciones al profesor en Plan de Riesgos (cliente/parte evaluadora); incluir reporte de auditoria F3
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -1937,8 +1937,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B7" s="31" t="inlineStr">
         <is>
-          <t>emitir notas tipificadas según mi rol (instrucción, acuerdo, solicitud, confirmación, respuesta) conforme al art. 125 RLOPSRM, con folio automático y firma electrónica</t>
+          <t>emitir notas tipificadas según mi rol —el residente autoriza y aprueba, el superintendente solicita y avisa, y la supervisión registra el avance— conforme al art. 125 RLOPSRM, con folio automático y firma electrónica</t>
         </is>
       </c>
       <c r="C7" s="32" t="n"/>
@@ -2442,8 +2442,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2685,8 +2685,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3190,8 +3190,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3433,8 +3433,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3938,8 +3938,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4181,8 +4181,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4690,8 +4690,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4933,8 +4933,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5438,8 +5438,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6336,8 +6336,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6579,8 +6579,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6822,8 +6822,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7065,8 +7065,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7308,8 +7308,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7551,8 +7551,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs: alinear criterios de historias con el sistema y actualizar estados a Terminado
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -1943,8 +1943,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>Solo aparecen disponibles los tipos de nota que corresponden al rol del usuario.</t>
+          <t>Solo aparecen los tipos de nota que corresponden al rol del usuario.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B14" s="36" t="inlineStr">
         <is>
-          <t>Cada nota queda registrada con folio, fecha, firmante y vínculo opcional a una nota previa.</t>
+          <t>Cada nota queda registrada con folio, fecha, firmante y vínculo opcional a nota previa.</t>
         </is>
       </c>
       <c r="C14" s="26" t="n"/>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -2454,8 +2454,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -2700,8 +2700,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>La carátula calcula automáticamente el anticipo amortizado (proporcional, art. 143 RLOPSRM), las retenciones legales (5 al millar, art. 191 LFD) y las deductivas por penalizaciones según el contrato.</t>
+          <t>La carátula calcula automáticamente anticipo amortizado, retenciones legales (5 al millar) y deductivas por penalizaciones según el contrato.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -2887,7 +2887,7 @@
       </c>
       <c r="B14" s="36" t="inlineStr">
         <is>
-          <t>El sistema bloquea la integración cuando una cantidad por concepto excede la cantidad contratada en el catálogo (art. 118 RLOPSRM: los trabajos por mayor valor sin orden escrita no son pagables).</t>
+          <t>El sistema bloquea la integración cuando una cantidad por concepto excede la cantidad contratada en el catálogo (art. 118 RLOPSRM).</t>
         </is>
       </c>
       <c r="C14" s="26" t="n"/>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -3211,8 +3211,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>La lista incluye todas las versiones (incluyendo rechazadas) con su periodo, estado e importe.</t>
+          <t>El historial muestra todas las estimaciones del contrato, incluyendo las versiones rechazadas.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>Solo existe una estimación con estado 'aceptada' por periodo, mientras que pueden existir múltiples rechazadas.</t>
+          <t>Por cada periodo solo puede haber una estimación aceptada; las versiones previas quedan marcadas como rechazadas.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -3457,8 +3457,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>La pantalla muestra todas las secciones de la estimación con posibilidad de registrar observaciones puntuales por sección.</t>
+          <t>La revisión permite revisar sección por sección y dejar observaciones puntuales en cada una (carátula, generadores, registro fotográfico, soportes y notas).</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>El flujo obliga a la supervisión a turnar la estimación antes de que residencia pueda autorizar o rechazar.</t>
+          <t>La autorización queda condicionada al turnado secuencial: primero supervisión, luego residencia; residencia no puede resolver antes del turnado.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="B14" s="36" t="inlineStr">
         <is>
-          <t>El sistema emite alertas cuando una estimación permanece más del plazo configurado en un mismo estado (art. 54 LOPSRM).</t>
+          <t>El sistema controla el plazo de 15 días naturales de revisión conforme al art. 54 LOPSRM mediante un semáforo visible para los actores.</t>
         </is>
       </c>
       <c r="C14" s="26" t="n"/>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -3968,8 +3968,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>El panel 'Mis pendientes' filtra los pendientes según el rol del usuario autenticado.</t>
+          <t>El panel "Mis pendientes" filtra los pendientes según el rol del usuario autenticado.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -4214,8 +4214,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4470,7 +4470,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -4728,8 +4728,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -4974,8 +4974,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>El sistema bloquea la instrucción de pago cuando la estimación excede el techo presupuestal disponible del contrato.</t>
+          <t>El sistema verifica suficiencia presupuestal contra el techo anual y bloquea la generación de la instrucción de pago si el monto excede lo disponible (art. 24 LOPSRM).</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -5143,7 +5143,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>El semáforo del plazo de pago (verde, ámbar, rojo) se calcula sobre los 20 días naturales y dispara alertas a Finanzas y Dependencia.</t>
+          <t>Un semáforo muestra el avance del plazo de 20 días naturales para pago (art. 54 LOPSRM) y emite alertas al entrar en amarillo.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B14" s="36" t="inlineStr">
         <is>
-          <t>La instrucción de pago se genera solo cuando todos los soportes obligatorios (factura, CFDI y, cuando aplique, estado de cuenta de fianza) están cargados.</t>
+          <t>La instrucción de pago solo puede generarse cuando todos los soportes obligatorios (factura, CFDI, estado de fianza) están cargados.</t>
         </is>
       </c>
       <c r="C14" s="26" t="n"/>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -5474,7 +5474,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -5485,8 +5485,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>Existe un contrato con folio único que contiene catálogo de conceptos, programa de obra, elementos jurídicos, garantías (anticipo, cumplimiento, vicios ocultos), penalizaciones aplicables, plan de amortización del anticipo y PDF firmado.</t>
+          <t>Existe un contrato con folio único que contiene catálogo de conceptos, programa de obra, elementos jurídicos, garantías, penalizaciones, plan de amortización del anticipo y PDF firmado.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>El sistema valida que los campos obligatorios estén llenos y el folio sea único antes de guardar; si falta alguno, no permite el guardado y señala el campo faltante.</t>
+          <t>El sistema valida que los campos obligatorios estén llenos y el folio sea único antes de guardar.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -6297,7 +6297,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>El sistema emite alerta cuando faltan N días configurables para el vencimiento de la póliza.</t>
+          <t>El sistema emite alerta cuando faltan N días configurables para el vencimiento.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -6377,7 +6377,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -6388,8 +6388,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -6634,8 +6634,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>La pantalla muestra los cinco bloques (configuración, catálogo, programa, fianzas, jurídicos) en una sola vista.</t>
+          <t>El expediente muestra en una sola vista los 5 bloques: configuración, catálogo, programa, fianzas y documentos jurídicos.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="B13" s="36" t="inlineStr">
         <is>
-          <t>El buscador permite filtrar por folio, contratista, objeto, periodo o tipo de documento.</t>
+          <t>El buscador filtra los bloques por folio, contratista, objeto, periodo o tipo de documento.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -6880,8 +6880,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -7126,8 +7126,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7361,7 +7361,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -7372,8 +7372,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -7618,8 +7618,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs: ajustar estados de historias a la realidad del sistema (HU-00 y HU-01 Terminado, resto En desarrollo)
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -1943,8 +1943,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -2454,8 +2454,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -2700,8 +2700,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -3211,8 +3211,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -3457,8 +3457,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -3968,8 +3968,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4203,7 +4203,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -4214,8 +4214,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -4728,8 +4728,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -4974,8 +4974,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="B20" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C20" s="34" t="n"/>
@@ -5474,7 +5474,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -5485,8 +5485,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6377,7 +6377,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -6388,8 +6388,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6623,7 +6623,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -6634,8 +6634,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6869,7 +6869,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -6880,8 +6880,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7115,7 +7115,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -7126,8 +7126,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7361,7 +7361,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -7372,8 +7372,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7607,7 +7607,7 @@
       </c>
       <c r="B19" s="37" t="inlineStr">
         <is>
-          <t>Terminado</t>
+          <t>En desarrollo</t>
         </is>
       </c>
       <c r="C19" s="34" t="n"/>
@@ -7618,8 +7618,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs: completar auditoría de las 22 HU (servicio SRV-00-01 + historias y servicios coherentes con el sistema)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -1725,7 +1725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -1765,6 +1765,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -1794,7 +1795,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>registrar por periodo las cantidades terminadas por cada concepto del catálogo, vinculando cada registro a su nota de bitácora del tipo Entrega</t>
+          <t>registrar por periodo las cantidades terminadas por cada concepto del catálogo, vinculando cada registro a su nota de bitácora del periodo, viendo el avance acumulado contra lo contratado en vivo</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -1814,6 +1815,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -1840,14 +1842,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Cada cantidad capturada queda ligada al concepto del catálogo correspondiente y a una nota de bitácora del periodo.</t>
+          <t>Cada cantidad capturada queda ligada al concepto del catálogo correspondiente y a una nota de bitácora del periodo (tipo entrega de obra o avance).</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -1858,14 +1858,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>El sistema bloquea el registro cuando la cantidad acumulada excede la contratada.</t>
+          <t>El sistema acumula el avance ejecutado por concepto y muestra el porcentaje de avance contra lo contratado en vivo, periodo a periodo.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -1875,35 +1873,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>El sistema bloquea el registro cuando la cantidad acumulada excede la contratada (art. 118 RLOPSRM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="n">
-        <v>3</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -1911,13 +1908,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="n">
+        <v>3</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -1925,24 +1920,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 7</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -1968,7 +1977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2008,6 +2017,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -2037,7 +2047,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>configurar qué conceptos del contrato quiero vigilar, el umbral de atraso a partir del cual quiero ser notificado y el canal de notificación</t>
+          <t>configurar qué conceptos del contrato quiero vigilar, el umbral de atraso a partir del cual quiero ser notificado y el canal de notificación (sistema o correo)</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -2057,6 +2067,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -2083,10 +2094,8 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
@@ -2101,14 +2110,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>El sistema solo dispara alertas cuando el avance real es menor al umbral configurado por el usuario.</t>
+          <t>La alerta solo dispara cuando el avance real es menor al umbral configurado por el usuario.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -2118,35 +2125,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>La notificación se entrega por el canal elegido al configurar la alerta (sistema o correo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="35" t="n">
-        <v>2</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -2154,13 +2160,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n">
+        <v>2</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -2168,24 +2172,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 6</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2251,7 +2269,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -2301,7 +2318,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -2375,7 +2391,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -2470,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -2510,6 +2525,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -2539,7 +2555,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>subir minutas de reuniones del contrato con sus metadatos, agendar visitas e inspecciones de campo, y consultar los acuerdos asentados</t>
+          <t>subir el PDF de las minutas de reuniones del contrato con sus metadatos, agendar visitas e inspecciones de campo, y consultar los acuerdos asentados, pudiendo adjuntar una minuta como referencia en una nota de bitácora</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -2559,6 +2575,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -2585,14 +2602,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Las minutas y visitas registradas son visibles para los usuarios autorizados del contrato.</t>
+          <t>Las minutas (con su PDF y metadatos) y las visitas registradas son visibles para los usuarios autorizados del contrato.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -2603,10 +2618,8 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
@@ -2620,35 +2633,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Una minuta o registro de visita puede adjuntarse como referencia en una nota de bitácora (HU-09).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="n">
-        <v>3</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -2656,13 +2668,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="n">
+        <v>3</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -2670,24 +2680,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 7</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2753,7 +2777,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -2803,7 +2826,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -2877,7 +2899,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -2972,7 +2993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3012,6 +3033,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3041,7 +3063,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>enviar formalmente una estimación integrada para que arranque el plazo de revisión del art. 54 LOPSRM</t>
+          <t>enviar formalmente una estimación integrada para que arranque el plazo de revisión del art. 54 LOPSRM, dentro de los 6 días naturales del periodo de presentación</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -3061,6 +3083,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3087,14 +3110,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Al enviar la estimación queda registrada la fecha y hora exacta, y se notifica a residencia y supervisión.</t>
+          <t>Al enviar la estimación quedan registradas la fecha y hora exacta de recepción, y queda notificación formal a residencia y supervisión.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -3105,10 +3126,8 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
@@ -3122,35 +3141,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Al enviarse, inicia automáticamente el plazo de revisión de 15 días naturales (supervisión, art. 54 LOPSRM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="n">
-        <v>3</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -3158,13 +3176,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 8</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="n">
+        <v>3</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -3172,24 +3188,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 8</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3215,7 +3245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3255,6 +3285,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3284,7 +3315,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>consultar todas las estimaciones del contrato a lo largo del tiempo con sus estados (aceptadas, rechazadas, en proceso) y filtros por periodo</t>
+          <t>consultar todas las estimaciones del contrato a lo largo del tiempo con sus estados (aceptadas, rechazadas, en proceso) y filtros por periodo, pudiendo abrir cada una para ver su expediente</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -3304,6 +3335,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3330,14 +3362,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>El historial muestra todas las estimaciones del contrato, incluyendo las versiones rechazadas.</t>
+          <t>El historial muestra todas las estimaciones del contrato en orden cronológico, incluyendo las versiones rechazadas.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -3348,14 +3378,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>Por cada periodo solo puede haber una estimación aceptada; las versiones previas quedan marcadas como rechazadas.</t>
+          <t>Los filtros permiten consultar por periodo, estado o ambos combinados (lógica Y).</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -3365,35 +3393,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cada estimación del historial puede abrirse para ver su expediente completo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="35" t="n">
-        <v>2</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -3401,13 +3428,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n">
+        <v>2</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -3415,24 +3440,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3498,6 +3537,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3527,7 +3567,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>revisar la estimación recibida sección por sección (carátula, números generadores, registro fotográfico, soportes, notas), registrar observaciones puntuales, turnar de supervisión a residencia y al final autorizar o rechazar</t>
+          <t>revisar la estimación recibida sección por sección (carátula, números generadores, registro fotográfico, soportes, notas), registrar observaciones con tipo y severidad, turnar de supervisión a residencia y al final autorizar o rechazar</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -3547,6 +3587,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3573,14 +3614,12 @@
       </c>
     </row>
     <row r="12" ht="33" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>La revisión permite revisar sección por sección y dejar observaciones puntuales en cada una (carátula, generadores, registro fotográfico, soportes y notas).</t>
+          <t>La revisión permite ir sección por sección (carátula, generadores, registro fotográfico, soportes y notas) y registrar observaciones con tipo y severidad por concepto.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -3591,10 +3630,8 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
@@ -3609,14 +3646,12 @@
       </c>
     </row>
     <row r="14" ht="33" customHeight="1" s="28">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A14" s="13" t="n">
+        <v>3</v>
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>El sistema controla el plazo de 15 días naturales de revisión conforme al art. 54 LOPSRM mediante un semáforo visible para los actores.</t>
+          <t>El sistema controla el plazo de 15 días naturales de revisión conforme al art. 54 LOPSRM mediante un semáforo basado en la fecha real de recepción.</t>
         </is>
       </c>
       <c r="C14" s="26" t="n"/>
@@ -3626,6 +3661,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -3720,7 +3756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -3760,6 +3796,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3809,6 +3846,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3835,10 +3873,8 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
@@ -3853,10 +3889,8 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
@@ -3870,35 +3904,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>La nueva versión queda vinculada con la rechazada para trazabilidad, sin reiniciar el plazo de presentación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="n">
-        <v>3</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -3906,13 +3939,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 8</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="n">
+        <v>3</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -3920,24 +3951,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 8</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3963,7 +4008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -4003,6 +4048,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -4032,7 +4078,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>ver en un tablero las estimaciones del contrato que están aceptadas y las que están en proceso (presentada, en revisión, autorizada, en pago, pagada), con su línea de tiempo y pendientes por solventar</t>
+          <t>ver en un tablero las estimaciones del contrato aceptadas y en proceso (presentada, en revisión, autorizada, en pago, pagada), con su línea de tiempo, indicadores y pendientes por solventar</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -4052,6 +4098,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -4078,10 +4125,8 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
@@ -4096,14 +4141,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>El panel "Mis pendientes" filtra los pendientes según el rol del usuario autenticado.</t>
+          <t>Cada estimación muestra su línea de tiempo de estado, y el tablero da indicadores agregados del contrato (avance, montos, días en cada estado).</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -4113,35 +4156,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>El panel «Mis pendientes» filtra los pendientes según el rol del usuario autenticado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="42" t="n">
-        <v>3</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -4149,13 +4191,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 8</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="n">
+        <v>3</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -4163,24 +4203,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 8</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4472,7 +4526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -4512,6 +4566,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -4561,6 +4616,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -4587,14 +4643,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Cada contrato del portafolio muestra un semáforo de color calculado a partir de avance físico, atrasos y pendientes.</t>
+          <t>Cada contrato del portafolio muestra un semáforo de color calculado a partir de tres factores: avance físico vs programado, atrasos en plazos legales y pendientes sin atender.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -4605,14 +4659,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>Al hacer doble clic sobre un contrato se abre su detalle con indicadores físicos, financieros y penalizaciones.</t>
+          <t>Al hacer doble clic sobre un contrato se abre su detalle con indicadores físicos, financieros, atrasos y penalizaciones.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -4622,35 +4674,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>El portafolio puede agruparse (por contratista, ejercicio fiscal o tipo de contratación) y comparar el periodo actual contra el anterior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="41" t="n">
-        <v>5</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -4658,13 +4709,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 9</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="n">
+        <v>5</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -4672,24 +4721,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 9</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4755,6 +4818,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -4804,6 +4868,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -4830,14 +4895,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Cada uno de los 7 reportes definidos genera el archivo en el formato establecido (PDF, Excel o ambos).</t>
+          <t>Cada uno de los 7 reportes definidos genera un archivo descargable en el formato establecido (PDF, Excel o ambos según el reporte).</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -4848,10 +4911,8 @@
       </c>
     </row>
     <row r="13" ht="33" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
@@ -4865,6 +4926,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="24" customHeight="1" s="28">
       <c r="A15" s="29" t="inlineStr">
         <is>
@@ -4931,8 +4993,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4998,6 +5060,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -5047,6 +5110,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -5073,10 +5137,8 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
@@ -5091,14 +5153,12 @@
       </c>
     </row>
     <row r="13" ht="33.9" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>Un semáforo muestra el avance del plazo de 20 días naturales para pago (art. 54 LOPSRM) y emite alertas al entrar en amarillo.</t>
+          <t>Un semáforo muestra el avance del plazo de 20 días naturales para pago (art. 54 LOPSRM), basado en la fecha de autorización, y avisa al entrar en amarillo.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -5109,14 +5169,12 @@
       </c>
     </row>
     <row r="14" ht="36.9" customHeight="1" s="28">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A14" s="13" t="n">
+        <v>3</v>
       </c>
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t>La instrucción de pago solo puede generarse cuando todos los soportes obligatorios (factura, CFDI, estado de fianza) están cargados.</t>
+          <t>La instrucción de pago solo puede generarse cuando todos los soportes obligatorios (factura, CFDI, estado de fianza de cumplimiento cuando el contrato lo exija) están cargados.</t>
         </is>
       </c>
       <c r="C14" s="26" t="n"/>
@@ -5126,6 +5184,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -5436,8 +5495,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5894,7 +5953,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -5944,7 +6002,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6018,7 +6075,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -6153,6 +6209,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6182,7 +6239,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>subir las pólizas de fianza del contrato (cumplimiento, vicios ocultos, anticipo) con sus metadatos: vigencia, afianzadora y monto afianzado</t>
+          <t>subir las pólizas de fianza del contrato (cumplimiento, vicios ocultos, anticipo) con sus metadatos (vigencia, afianzadora y monto), recibir alertas anticipadas de vencimiento y mantener el historial de fianzas y sus endosos por modificatorios</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -6202,6 +6259,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6228,10 +6286,8 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
@@ -6246,14 +6302,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>El sistema emite alerta cuando faltan N días configurables para el vencimiento.</t>
+          <t>El sistema emite alerta cuando faltan 30, 15 y 5 días para el vencimiento (configurable).</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -6344,8 +6398,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6371,7 +6425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -6411,6 +6465,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6440,7 +6495,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>registrar un convenio modificatorio del contrato (cambios al monto, plazo o conceptos) y aplicar las actualizaciones al catálogo, programa y fianzas, manteniendo el histórico de versiones</t>
+          <t>registrar un convenio modificatorio del contrato (cambios al monto, plazo o conceptos) y aplicar las actualizaciones al catálogo, programa y endosos de las fianzas, manteniendo el histórico de versiones conforme al art. 59 LOPSRM</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -6460,6 +6515,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6486,14 +6542,12 @@
       </c>
     </row>
     <row r="12" ht="33" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>Al autorizarse el modificatorio se generó una nueva versión del catálogo y del programa, sin alterar la versión anterior.</t>
+          <t>Al registrarse el modificatorio se genera una nueva versión del catálogo y del programa, sin alterar la versión anterior.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -6504,14 +6558,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>El histórico de versiones registra fecha, autor y motivo del cambio para cada modificatorio.</t>
+          <t>El sistema indica si el modificatorio se rige por el art. 59 LOPSRM (modificatorio ordinario) o por el art. 59 Bis (ajuste de costos cuando se supera 50% del monto o 50% del plazo).</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -6521,35 +6573,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>El histórico de versiones registra fecha, autor y motivo del cambio, y los endosos correspondientes a las fianzas asociadas al modificatorio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="41" t="n">
-        <v>5</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -6557,13 +6608,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 6</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="n">
+        <v>5</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -6571,24 +6620,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 6</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6614,7 +6677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="16" customWidth="1" style="28" min="1" max="1"/>
@@ -6654,6 +6717,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6683,7 +6747,7 @@
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>consultar en una sola vista todos los elementos vigentes del contrato (configuración, catálogo, programa, fianzas, elementos jurídicos) con buscador</t>
+          <t>consultar en una sola vista los 5 bloques vigentes del contrato (configuración, catálogo, programa, fianzas y documentos jurídicos), con buscador combinable y descarga individual de documentos</t>
         </is>
       </c>
       <c r="C7" s="31" t="n"/>
@@ -6703,6 +6767,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6729,14 +6794,12 @@
       </c>
     </row>
     <row r="12" ht="32.1" customHeight="1" s="28">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A12" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="25" t="inlineStr">
         <is>
-          <t>El expediente muestra en una sola vista los 5 bloques: configuración, catálogo, programa, fianzas y documentos jurídicos.</t>
+          <t>El expediente muestra en una sola vista los 5 bloques del contrato: configuración, catálogo, programa, fianzas y documentos jurídicos.</t>
         </is>
       </c>
       <c r="C12" s="26" t="n"/>
@@ -6747,14 +6810,12 @@
       </c>
     </row>
     <row r="13" ht="32.1" customHeight="1" s="28">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="A13" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="25" t="inlineStr">
         <is>
-          <t>El buscador filtra los bloques por folio, contratista, objeto, periodo o tipo de documento.</t>
+          <t>El buscador filtra los bloques por folio, contratista, objeto, periodo o tipo de documento, con lógica Y.</t>
         </is>
       </c>
       <c r="C13" s="26" t="n"/>
@@ -6764,35 +6825,34 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" s="28">
-      <c r="A15" s="29" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cada documento del expediente puede descargarse individualmente desde su bloque.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="28"/>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>METADATOS DE PLANEACIÓN (Scrum)</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="28">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Complejidad</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="26" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1" s="28">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
-        </is>
-      </c>
-      <c r="B17" s="35" t="n">
-        <v>2</v>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
       </c>
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="26" t="n"/>
@@ -6800,13 +6860,11 @@
     <row r="18" ht="24" customHeight="1" s="28">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Sprint propuesto</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n">
+        <v>2</v>
       </c>
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="26" t="n"/>
@@ -6814,24 +6872,38 @@
     <row r="19" ht="24" customHeight="1" s="28">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Sprint propuesto</t>
         </is>
       </c>
       <c r="B19" s="30" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6897,7 +6969,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6947,7 +7018,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -7082,8 +7152,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7149,7 +7219,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -7199,7 +7268,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -7334,8 +7402,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7401,7 +7469,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -7451,7 +7518,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -7509,7 +7575,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="24" customHeight="1" s="28">
       <c r="A15" s="29" t="inlineStr">
         <is>
@@ -7576,8 +7641,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>

<commit_message>
docs: agregar historia de registro a historias de usuario
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Historias_Usuario.xlsx
+++ b/docs/Historias_Usuario.xlsx
@@ -29,8 +29,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HU-19" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HU-20" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HU-21" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan_Iteraciones" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan_Iteraciones" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -698,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" style="28" min="1" max="1"/>
@@ -1698,6 +1699,44 @@
       <c r="H31" s="5" t="inlineStr">
         <is>
           <t>Sprint 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="27.9" customHeight="1" s="28">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Registro</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Registro de usuario con aprobación</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Control de Accesos</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Usuario nuevo / Dependencia</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Agregada tras la revisión</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1804,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -1815,7 +1853,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -1950,8 +1987,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2017,7 +2054,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -2067,7 +2103,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -2202,8 +2237,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -2525,7 +2560,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -2575,7 +2609,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -2710,8 +2743,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3033,7 +3066,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3083,7 +3115,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3218,8 +3249,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3285,7 +3316,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3335,7 +3365,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3470,8 +3499,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -3537,7 +3566,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3587,7 +3615,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3661,7 +3688,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -3796,7 +3822,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -3846,7 +3871,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -3981,8 +4005,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4048,7 +4072,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -4098,7 +4121,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -4233,8 +4255,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4566,7 +4588,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -4616,7 +4637,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -4751,8 +4771,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -4818,7 +4838,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -4868,7 +4887,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -4926,7 +4944,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="24" customHeight="1" s="28">
       <c r="A15" s="29" t="inlineStr">
         <is>
@@ -4993,8 +5010,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5060,7 +5077,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -5110,7 +5126,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -5184,7 +5199,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="24" customHeight="1" s="28">
       <c r="A16" s="29" t="inlineStr">
         <is>
@@ -5495,8 +5509,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -5522,6 +5536,270 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="16" customWidth="1" style="28" min="1" max="1"/>
+    <col width="50" customWidth="1" style="28" min="2" max="2"/>
+    <col width="25" customWidth="1" style="28" min="3" max="3"/>
+    <col width="18" customWidth="1" style="28" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1" s="28">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>Registro · Registro de usuario con aprobación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="28">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>Servicio implementado: Control de Accesos</t>
+        </is>
+      </c>
+      <c r="C2" s="32" t="inlineStr">
+        <is>
+          <t>Módulo: —</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" s="28">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Sprint sugerido: Agregada tras la revisión</t>
+        </is>
+      </c>
+      <c r="C3" s="32" t="inlineStr">
+        <is>
+          <t>Estado: Backlog</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" s="28">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>HISTORIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27.9" customHeight="1" s="28">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>usuario nuevo</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="n"/>
+      <c r="D6" s="26" t="n"/>
+    </row>
+    <row r="7" ht="69" customHeight="1" s="28">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Deseo</t>
+        </is>
+      </c>
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>registrarme en el sistema proporcionando mis datos</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="26" t="n"/>
+    </row>
+    <row r="8" ht="27.9" customHeight="1" s="28">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>A fin de</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>solicitar acceso y que la dependencia valide mi identidad y asigne mi rol</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="n"/>
+      <c r="D8" s="26" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1" s="28">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>CRITERIOS DE ACEPTACIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>Criterios de aceptación</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>Resultado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32.1" customHeight="1" s="28">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>El registro captura los datos del solicitante y crea la cuenta en estado pendiente, sin otorgar acceso.</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>☐ Sí   ☐ No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32.1" customHeight="1" s="28">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>El sistema impide el ingreso de cuentas no aprobadas e informa que están pendientes de autorización.</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n"/>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>☐ Sí   ☐ No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32.1" customHeight="1" s="28">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>La dependencia revisa las solicitudes, asigna el rol y aprueba o rechaza; solo las cuentas aprobadas pueden ingresar.</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>☐ Sí   ☐ No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="n"/>
+      <c r="B15" s="25" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="28">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>METADATOS DE PLANEACIÓN (Scrum)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" s="28">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Complejidad</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="28">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>User points (Fibonacci 1, 2, 3, 5, 8)</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="26" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="28">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Sprint propuesto</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Agregada tras la revisión</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="26" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="28">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Terminado</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="26" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="C3:D3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -5894,7 +6172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6209,7 +6487,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6259,7 +6536,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6398,8 +6674,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6465,7 +6741,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6515,7 +6790,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6650,8 +6924,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -6717,7 +6991,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="28">
       <c r="A5" s="29" t="inlineStr">
         <is>
@@ -6767,7 +7040,6 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="26" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="28">
       <c r="A10" s="29" t="inlineStr">
         <is>
@@ -6902,8 +7174,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7152,8 +7424,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7402,8 +7674,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>
@@ -7641,8 +7913,8 @@
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B6:D6"/>

</xml_diff>